<commit_message>
fix: secure rule pack publishing
</commit_message>
<xml_diff>
--- a/rules/templates/security-review-rules-template.xlsx
+++ b/rules/templates/security-review-rules-template.xlsx
@@ -7,18 +7,24 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detectors" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则包信息" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="敏感类别" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产专项规则" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="受限实体词典" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="安全占位符" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检测器配置" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第三方授权" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合规规则" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Categories'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assets'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRules'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rules'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Detectors'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'规则包信息'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'敏感类别'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'资产专项规则'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'受限实体词典'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'安全占位符'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'检测器配置'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'第三方授权'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'合规规则'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,79 +451,111 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CategoryId</t>
+          <t>键</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Enabled</t>
+          <t>值</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SENS-001</t>
+          <t>rulePackId</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Sensitive Personal Data</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Scan for PII, credentials, and tokens</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="b">
-        <v>1</v>
+          <t>security-review-rules</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>SENS-002</t>
+          <t>version</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Access Control</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Detect improper ACLs and permissions</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="b">
-        <v>1</v>
+          <t>1.0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>schemaVersion</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>minClientVersion</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>createdAtUtc</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24T00:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>signerKeyId</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>rules-team-prod-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>changeSummary</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>请填写本次规则变更说明</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -528,61 +566,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AssetTypeId</t>
+          <t>类别ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>名称</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>说明</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>FocusWeights</t>
+          <t>默认严重度</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>启用</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ASSET-001</t>
+          <t>SENS-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Source Code Repository</t>
+          <t>凭据和密钥</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Git repositories containing application source code</t>
+          <t>API 密钥、密码和访问令牌</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>{"SENS-001": 1.0, "SENS-002": 0.5}</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -593,53 +642,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>规则ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>AssetTypeId</t>
+          <t>资产ID</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>类别ID</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>发现类型</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>EvidenceField</t>
+          <t>检测器ID</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>RequiredStatus</t>
+          <t>配置ID</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>严重度</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>置信度</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>需要语义复核</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>启用</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CR-SOURCE-001</t>
+          <t>RULE-TEMPLATE-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -649,27 +728,52 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>GitHub Branch Protection</t>
+          <t>SENS-001</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Verify branch protection rules are enabled for the default branch</t>
+          <t>SensitiveContent</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>branch_protection</t>
+          <t>DET-TEMPLATE-001</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>示例规则，请按实际需要修改</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -680,123 +784,116 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RuleId</t>
+          <t>词典ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>CategoryId</t>
+          <t>实体ID</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>FindingKind</t>
+          <t>标准名称</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Severity</t>
+          <t>变体</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>DetectionConfidence</t>
+          <t>类别ID</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>DetectorId</t>
+          <t>严重度</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>DetectorConfigId</t>
+          <t>资产范围</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>AppliesToAssets</t>
+          <t>有效起始</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>RequiresSemanticReview</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Enabled</t>
+          <t>有效结束</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RULE-AWS-KEY-001</t>
+          <t>dict-template</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>entity-template</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>示例受限实体</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>示例别名</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>SENS-001</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>SensitiveContent</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>DET-CRED-001</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>aws-access-key</t>
+          <t>ASSET-001</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>ASSET-001,ASSET-002</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2" t="b">
-        <v>1</v>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -807,70 +904,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DetectorId</t>
+          <t>占位符ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Kind</t>
+          <t>匹配类型</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ConfigId</t>
+          <t>值</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Parameters</t>
+          <t>允许上下文</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>MaxMatchesPerChunk</t>
+          <t>类别ID</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>有效起始</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>有效结束</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DET-CRED-001</t>
+          <t>placeholder-template</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>regex</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>example_placeholder</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>SENS-001</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>检测器ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>配置ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>参数JSON</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>最大每块命中数</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DET-TEMPLATE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>KnownFormat</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>aws-access-key</t>
+          <t>default</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>{"pattern": "AKIA[0-9A-Z]{16}", "description": "AWS Access Key ID"}</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>100</v>
+          <t>{"format":"pem"}</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>授权ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>来源名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>标识或指纹</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>许可说明</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>证据引用</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>有效起始</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>有效结束</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>license-template</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>示例依赖</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>example-fingerprint</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.invalid/license</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>规则ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>资产ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>证据字段</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>缺失结论</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>严重度</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>COMP-TEMPLATE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ASSET-001</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>evidence.json</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>示例合规规则，请按实际需要修改</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>